<commit_message>
Remove stray table borders from summary Excel template and count old records based on 2 fiscal years
</commit_message>
<xml_diff>
--- a/dist/summary-template.xlsx
+++ b/dist/summary-template.xlsx
@@ -83,7 +83,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -118,14 +118,6 @@
       <name val="TH SarabunIT๙"/>
     </font>
     <font>
-      <charset val="222"/>
-      <color theme="1"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
       <b/>
       <color theme="1"/>
       <family val="2"/>
@@ -147,7 +139,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -207,31 +199,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -279,9 +251,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -324,32 +293,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -689,13 +645,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD173"/>
+  <dimension ref="A1:AN173"/>
   <sheetFormatPr defaultRowHeight="16.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="4" max="4" width="29.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="22.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -707,7 +663,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
     </row>
-    <row r="2" ht="12" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="12" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -717,7 +673,7 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" ht="19.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="19.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -731,7 +687,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
     </row>
-    <row r="4" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -749,7 +705,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" ht="23.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="23.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -761,7 +717,7 @@
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" ht="21" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="21" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
@@ -781,7 +737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>9</v>
       </c>
@@ -801,7 +757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="18.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="18.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>10</v>
       </c>
@@ -821,7 +777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="21" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="21" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>11</v>
       </c>
@@ -841,7 +797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="18.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="18.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>12</v>
       </c>
@@ -861,7 +817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="21" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="21" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>13</v>
       </c>
@@ -881,7 +837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="39.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="39.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>14</v>
       </c>
@@ -893,7 +849,7 @@
       <c r="G12" s="13"/>
       <c r="H12" s="14"/>
     </row>
-    <row r="13" ht="37.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="37.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="str">
         <f>'[1]รายเก่า รายใหม่'!A14</f>
         <v>(1) การฆ่า หรือชำแหละสัตว์ ยกเว้นในสถานที่จำหน่ายอาหาร เร่ขาย หรือขายในตลาด</v>
@@ -914,7 +870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A14" s="16" t="str">
         <f>'[1]รายเก่า รายใหม่'!A15</f>
         <v>(2) การหมัก ฟอก ตาก หรือสะสมหนังสัตว์ ขนสัตว์</v>
@@ -935,7 +891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="19.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="19.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="str">
         <f>'[1]รายเก่า รายใหม่'!A16</f>
         <v>(3) การสะสมเขา กระดูก หรือชิ้นส่วนสัตว์ที่ยังมิได้แปรรูป</v>
@@ -956,7 +912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="21" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="21" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A16" s="16" t="str">
         <f>'[1]รายเก่า รายใหม่'!A17</f>
         <v>(4) การเคี่ยวหนัง เอ็น หรือไขสัตว์</v>
@@ -977,7 +933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="57" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="57" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="str">
         <f>'[1]รายเก่า รายใหม่'!A18</f>
         <v>(5) การผลิตสิ่งของเครื่องใช้หรือผลิตภัณฑ์อื่น ๆ จากเปลือก กระดอง กระดูก เขา หนัง ขนสัตว์หรือส่วนอื่น ๆ ของสัตว์ด้วยการต้ม นึ่ง ตาก เผาหรือกรรมวิธีใด ๆ ซึ่งมิใช่เพื่อเป็นอาหาร</v>
@@ -996,7 +952,7 @@
       </c>
       <c r="H17" s="8"/>
     </row>
-    <row r="18" ht="57.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="57.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="str">
         <f>'[1]รายเก่า รายใหม่'!A19</f>
         <v>(6) การผลิต โม่ ป่น บด ผสม บรรจุ สะสม หรือกระทำอื่นใดต่อสัตว์หรือพืช หรือส่วนหนึ่งส่วนใดของสัตว์หรือพืชเพื่อเป็นอาหารสัตว์หรือส่วนประกอบของอาหารสัตว์</v>
@@ -1017,7 +973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="str">
         <f>'[1]รายเก่า รายใหม่'!A20</f>
         <v>(7) การผลิต แปรรูป สะสม หรือล้างครั่ง</v>
@@ -1037,22 +993,20 @@
       <c r="H19" s="8">
         <v>0</v>
       </c>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-    </row>
-    <row r="20" ht="41.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A20" s="18" t="s">
+    </row>
+    <row r="20" ht="41.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-    </row>
-    <row r="21" ht="38.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+    </row>
+    <row r="21" ht="38.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="str">
         <f>'[1]รายเก่า รายใหม่'!A22</f>
         <v>(1) การผลิต สะสม หรือแบ่งบรรจุ น้ำพริกแกง น้ำพริกปรุงสำเร็จ เต้าเจี้ยว ซีอิ๊ว น้ำจิ้ม หรือซอสปรุงรสชนิดต่าง ๆ</v>
@@ -1073,7 +1027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" ht="55.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="55.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="str">
         <f>'[1]รายเก่า รายใหม่'!A23</f>
         <v>(2) การผลิต สะสม หรือแบ่งบรรจุ อาหารหมัก ดอง จากสัตว์ ได้แก่ ปลาร้า ปลาเจ่า กุ้งเจ่า ปลาส้ม ปลาจ่อม แหนม หม่ำ ไส้กรอก กะปิ น้ำปลา หอยดอง น้ำเคย น้ำบูดู ไตปลา หรือผลิตภัณฑ์อื่น ๆ ที่คล้ายคลึงกัน</v>
@@ -1094,7 +1048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="37.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="37.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="str">
         <f>'[1]รายเก่า รายใหม่'!A24</f>
         <v>(3) การผลิต สะสม หรือแบ่งบรรจุ อาหารหมัก ดอง แช่อิ่ม จากผัก ผลไม้ หรือพืชอย่างอื่น</v>
@@ -1115,7 +1069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" ht="39.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="39.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="str">
         <f>'[1]รายเก่า รายใหม่'!A25</f>
         <v>(4) การผลิต สะสม หรือแบ่งบรรจุ อาหารจากพืชหรือสตว์ โดยการตาก บด นึ่ง ต้ม ตุ๋น เคี่ยว กวน ฉาบ ทอด อบ รมควัน ปิ้ง ย่าง เผา หรือวิธีอื่นใด</v>
@@ -1136,14 +1090,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="22.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A25" s="20" t="str">
+    <row r="25" ht="22.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A25" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A26</f>
         <v>(5) การผลิต สะสม หรือแบ่งบรรจุลูกชิ้น</v>
       </c>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
       <c r="E25" s="8">
         <v>0</v>
       </c>
@@ -1157,14 +1111,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" ht="42" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="str">
+    <row r="26" ht="42" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A26" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A27</f>
         <v>(6) การผลิต สะสม หรือแบ่งบรรจุ เส้นหมี่ ขนมจีน ก๋วยเตี๋ยว เต้าฮวย เต้าหู้ วุ้นเส้น เกี้ยมอี๋ เนื้อสัตว์เทียม หรือผลิตภัณฑ์อื่น ๆ ที่คล้ายคลึงกัน</v>
       </c>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
       <c r="E26" s="8">
         <v>0</v>
       </c>
@@ -1178,7 +1132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>1</v>
       </c>
@@ -1192,7 +1146,7 @@
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
     </row>
-    <row r="28" ht="21.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1210,14 +1164,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" ht="21.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="str">
+    <row r="29" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A29" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A28</f>
         <v>(7) การผลิตบะหมี่ มักกะโรนี สปาเกตตี้ พาสตา หรือผลิตภัณฑ์อื่น ๆ ที่คล้ายคลึงกัน</v>
       </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
       <c r="E29" s="8">
         <v>0</v>
       </c>
@@ -1231,14 +1185,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A30" s="20" t="str">
+    <row r="30" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A30" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A29</f>
         <v>(8) การผลิต ขนมปังสด ขนมปังแห้ง จันอับ ขนมเปี๊ยะ ขนมอบอื่น ๆ</v>
       </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
       <c r="E30" s="8">
         <v>3</v>
       </c>
@@ -1252,14 +1206,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="21.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A31" s="20" t="str">
+    <row r="31" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A31" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A30</f>
         <v>(9) การผลิต สะสม หรือแบ่งบรรจุ น้ำนม หรือผลิตภัณฑ์จากน้ำนมสัตว์</v>
       </c>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
       <c r="E31" s="8">
         <v>1</v>
       </c>
@@ -1273,14 +1227,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" ht="39.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A32" s="21" t="str">
+    <row r="32" ht="39.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A32" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A31</f>
         <v>(10) การผลิต สะสม หรือแบ่งบรรจุ เนย เนยเทียม เนยผสม ผลิตภัณฑ์เนย ผลิตภัณฑ์เนยเทียม และผลิตภัณฑ์เนยผสม</v>
       </c>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
       <c r="E32" s="8">
         <v>0</v>
       </c>
@@ -1294,14 +1248,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" ht="24.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A33" s="20" t="str">
+    <row r="33" ht="24.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A33" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A32</f>
         <v>(11) การผลิตไอศกรีม</v>
       </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
       <c r="E33" s="8">
         <v>0</v>
       </c>
@@ -1315,14 +1269,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A34" s="20" t="str">
+    <row r="34" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A33</f>
         <v>(12) การคั่ว สะสม หรือแบ่งบรรจุกาแฟ</v>
       </c>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
       <c r="E34" s="8">
         <v>0</v>
       </c>
@@ -1336,14 +1290,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" ht="29.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A35" s="21" t="str">
+    <row r="35" ht="29.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A35" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A34</f>
         <v>(13) การผลิต สะสม หรือแบ่งบรรจุ ใบชาแห้ง ชาผง หรือเครื่องดื่มชนิดผงอื่น ๆ</v>
       </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
       <c r="E35" s="8">
         <v>0</v>
       </c>
@@ -1357,14 +1311,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" ht="39.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A36" s="21" t="str">
+    <row r="36" ht="39.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A36" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A35</f>
         <v>(14) การผลิต สะสม หรือแบ่งบรรจุ เอทิลแอลกอฮอล์ สุรา เบียร์ ไวน์ น้ำส้มสายชู ข้าวหมาก น้ำตาลเมา</v>
       </c>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
+      <c r="B36" s="19"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
       <c r="E36" s="8">
         <v>0</v>
       </c>
@@ -1378,14 +1332,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" ht="21.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A37" s="20" t="str">
+    <row r="37" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A37" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A36</f>
         <v>(15) การผลิตน้ำกลั่น น้ำบริโภค น้ำดื่มจากเครื่องจำหน่ายอัตโนมัติ</v>
       </c>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
+      <c r="B37" s="19"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
       <c r="E37" s="8">
         <v>0</v>
       </c>
@@ -1399,14 +1353,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" ht="21.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A38" s="20" t="str">
+    <row r="38" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A37</f>
         <v>(16) การผลิต สะสม แบ่งบรรจุ หรือขนส่งน้ำแข็ง</v>
       </c>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
       <c r="E38" s="8">
         <v>0</v>
       </c>
@@ -1420,14 +1374,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="42.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A39" s="21" t="str">
+    <row r="39" ht="42.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A39" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A38</f>
         <v>(17) การผลิต สะสม หรือแบ่งบรรจุ น้ำอัดลม น้ำหวาน น้ำโซดา น้ำจากพืช ผัก ผลไม้ เครื่องดื่มชนิดต่าง ๆ บรรจุกระป๋อง ขวดหรือภาชนะอื่นใด</v>
       </c>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
       <c r="E39" s="8">
         <v>0</v>
       </c>
@@ -1441,14 +1395,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" ht="24.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A40" s="21" t="str">
+    <row r="40" ht="24.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A40" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A39</f>
         <v>(18) การผลิต สะสม หรือแบ่งบรรจุ อาหารบรรจุกระป๋อง ขวด หรือภาชนะอื่นใด</v>
       </c>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
       <c r="E40" s="8">
         <v>4</v>
       </c>
@@ -1462,98 +1416,98 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" ht="24.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A41" s="20" t="str">
+    <row r="41" ht="24.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A41" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A40</f>
         <v>(19) การผลิต สะสม หรือแบ่งบรรจุ ผงชูรส หรือสารปรุงแต่งอาหาร</v>
       </c>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="22">
-        <v>0</v>
-      </c>
-      <c r="F41" s="22">
-        <v>0</v>
-      </c>
-      <c r="G41" s="22">
-        <v>0</v>
-      </c>
-      <c r="H41" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" ht="27" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A42" s="20" t="str">
+      <c r="B41" s="19"/>
+      <c r="C41" s="19"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="21">
+        <v>0</v>
+      </c>
+      <c r="F41" s="21">
+        <v>0</v>
+      </c>
+      <c r="G41" s="21">
+        <v>0</v>
+      </c>
+      <c r="H41" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" ht="27" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A42" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A41</f>
         <v>(20) การผลิต สะสม หรือแบ่งบรรจุ น้ำตาล น้ำเชื่อม</v>
       </c>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="22">
-        <v>0</v>
-      </c>
-      <c r="F42" s="22">
-        <v>0</v>
-      </c>
-      <c r="G42" s="22">
-        <v>0</v>
-      </c>
-      <c r="H42" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A43" s="20" t="str">
+      <c r="B42" s="19"/>
+      <c r="C42" s="19"/>
+      <c r="D42" s="19"/>
+      <c r="E42" s="21">
+        <v>0</v>
+      </c>
+      <c r="F42" s="21">
+        <v>0</v>
+      </c>
+      <c r="G42" s="21">
+        <v>0</v>
+      </c>
+      <c r="H42" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A42</f>
         <v>(21) การผลิต สะสม หรือแบ่งบรรจุแบะแซ</v>
       </c>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="22">
-        <v>0</v>
-      </c>
-      <c r="F43" s="22">
-        <v>0</v>
-      </c>
-      <c r="G43" s="22">
-        <v>0</v>
-      </c>
-      <c r="H43" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" ht="28.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A44" s="21" t="str">
+      <c r="B43" s="19"/>
+      <c r="C43" s="19"/>
+      <c r="D43" s="19"/>
+      <c r="E43" s="21">
+        <v>0</v>
+      </c>
+      <c r="F43" s="21">
+        <v>0</v>
+      </c>
+      <c r="G43" s="21">
+        <v>0</v>
+      </c>
+      <c r="H43" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="28.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A44" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A43</f>
         <v>(22) การแกะ ตัดแต่ง ล้างสัตว์น้ำ ที่ไม่ใช่เป็นส่วนหนึ่งของกิจการห้องเย็น</v>
       </c>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="22">
-        <v>0</v>
-      </c>
-      <c r="F44" s="22">
-        <v>0</v>
-      </c>
-      <c r="G44" s="22">
-        <v>0</v>
-      </c>
-      <c r="H44" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" ht="22.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A45" s="20" t="str">
+      <c r="B44" s="19"/>
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="21">
+        <v>0</v>
+      </c>
+      <c r="F44" s="21">
+        <v>0</v>
+      </c>
+      <c r="G44" s="21">
+        <v>0</v>
+      </c>
+      <c r="H44" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="22.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A45" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A44</f>
         <v>(23) การประกอบกิจการห้องเย็นแช่แข็งอาหาร</v>
       </c>
-      <c r="B45" s="20"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
+      <c r="B45" s="19"/>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
       <c r="E45" s="8">
         <v>1</v>
       </c>
@@ -1567,14 +1521,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" ht="21.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A46" s="20" t="str">
+    <row r="46" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A46" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A45</f>
         <v>(24) การเก็บ การถนอมอาหารด้วยเครื่องจักร</v>
       </c>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
+      <c r="B46" s="19"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
       <c r="E46" s="8">
         <v>1</v>
       </c>
@@ -1587,31 +1541,27 @@
       <c r="H46" s="8">
         <v>0</v>
       </c>
-      <c r="I46" s="17"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
-    </row>
-    <row r="47" ht="25.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A47" s="23" t="s">
+    </row>
+    <row r="47" ht="25.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A47" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B47" s="24"/>
-      <c r="C47" s="24"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
-      <c r="G47" s="24"/>
-      <c r="H47" s="25"/>
-    </row>
-    <row r="48" ht="22.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A48" s="20" t="str">
+      <c r="B47" s="23"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="24"/>
+    </row>
+    <row r="48" ht="22.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A48" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A47</f>
         <v>(1) การผลิต โม่ บด ผสม หรือบรรจุยา</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="19"/>
+      <c r="D48" s="19"/>
       <c r="E48" s="8">
         <v>0</v>
       </c>
@@ -1625,14 +1575,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" ht="39" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A49" s="21" t="str">
+    <row r="49" ht="39" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A49" s="20" t="str">
         <f>'[1]รายเก่า รายใหม่'!A48</f>
         <v>(2) การผลิต บรรจุยาสีฟัน แชมพู ผ้าเย็น กระดาษเย็น เครื่องสำอาง รวมทั้งสบู่ที่ใช้กับร่างกาย</v>
       </c>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
+      <c r="B49" s="19"/>
+      <c r="C49" s="19"/>
+      <c r="D49" s="19"/>
       <c r="E49" s="8">
         <v>3</v>
       </c>
@@ -1646,14 +1596,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A50" s="20" t="str">
+    <row r="50" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A50" s="19" t="str">
         <f>'[1]รายเก่า รายใหม่'!A49</f>
         <v>(3) การผลิต บรรจุสำลี ผลิตภัณฑ์จากสำลี</v>
       </c>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
+      <c r="B50" s="19"/>
+      <c r="C50" s="19"/>
+      <c r="D50" s="19"/>
       <c r="E50" s="8">
         <v>0</v>
       </c>
@@ -1667,7 +1617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A50</f>
         <v>(4) การผลิตผ้าพันแผล ผ้าปิดแผล ผ้าอนามัย ผ้าอ้อมสำเร็จรูป</v>
@@ -1688,8 +1638,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" ht="32.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A52" s="26" t="str">
+    <row r="52" ht="32.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A52" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A51</f>
         <v>(5) การผลิตผงซักฟอก สบู่ น้ำยาทำความสะอาด หรือผลิตภัณฑ์ทำความสะอาดต่าง ๆ</v>
       </c>
@@ -1708,22 +1658,20 @@
       <c r="H52" s="8">
         <v>0</v>
       </c>
-      <c r="I52" s="17"/>
-      <c r="J52" s="17"/>
-    </row>
-    <row r="53" ht="28.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A53" s="23" t="s">
+    </row>
+    <row r="53" ht="28.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A53" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B53" s="24"/>
-      <c r="C53" s="24"/>
-      <c r="D53" s="24"/>
-      <c r="E53" s="24"/>
-      <c r="F53" s="24"/>
-      <c r="G53" s="24"/>
-      <c r="H53" s="25"/>
-    </row>
-    <row r="54" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B53" s="23"/>
+      <c r="C53" s="23"/>
+      <c r="D53" s="23"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="23"/>
+      <c r="G53" s="23"/>
+      <c r="H53" s="24"/>
+    </row>
+    <row r="54" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A53</f>
         <v>(1) การผลิต สะสม หรือแบ่งบรรจุน้ำมันจากพืช</v>
@@ -1731,21 +1679,21 @@
       <c r="B54" s="10"/>
       <c r="C54" s="10"/>
       <c r="D54" s="11"/>
-      <c r="E54" s="22">
-        <v>0</v>
-      </c>
-      <c r="F54" s="22">
-        <v>0</v>
-      </c>
-      <c r="G54" s="22">
-        <v>0</v>
-      </c>
-      <c r="H54" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" ht="22.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A55" s="26" t="str">
+      <c r="E54" s="21">
+        <v>0</v>
+      </c>
+      <c r="F54" s="21">
+        <v>0</v>
+      </c>
+      <c r="G54" s="21">
+        <v>0</v>
+      </c>
+      <c r="H54" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" ht="22.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A55" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A54</f>
         <v>(2) การล้าง อบ รม หรือสะสมยางดิบ</v>
       </c>
@@ -1765,7 +1713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" ht="22.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="22.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A55</f>
         <v>(3) การผลิต หรือแบ่งบรรจุแป้งมันสำปะหลัง แป้งสาคู แป้งจากพืช หรือแป้งอื่น ๆ ในทำนองเดียวกัน</v>
@@ -1786,7 +1734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" ht="24.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="24.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>1</v>
       </c>
@@ -1800,7 +1748,7 @@
       <c r="G57" s="3"/>
       <c r="H57" s="3"/>
     </row>
-    <row r="58" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -1818,7 +1766,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A56</f>
         <v>(4) การสีข้าว นวดข้าวด้วยเครื่องจักร หรือแบ่งบรรจุข้าวด้วยวิธีใด ๆ ก็ตาม</v>
@@ -1839,7 +1787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A57</f>
         <v>(5) การผลิตยาสูบ</v>
@@ -1860,7 +1808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A58</f>
         <v>(6) การขัด กะเทาะ หรือบดเมล็ดพืช</v>
@@ -1881,7 +1829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A59</f>
         <v>(7) การผลิต สะสม หรือแบ่งบรรจุปุ๋ยหรือวัสดุที่นำไปผลิตปุ๋ย</v>
@@ -1902,7 +1850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A60</f>
         <v>(8) การผลิตเส้นใยจากพืช</v>
@@ -1923,8 +1871,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" ht="21.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A64" s="26" t="str">
+    <row r="64" ht="21.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A64" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A61</f>
         <v>(9) การตาก สะสม ขนถ่ายผลิตผลของมันสำปะหลัง ข้าวเปลือก อ้อย ข้าวโพด</v>
       </c>
@@ -1943,29 +1891,27 @@
       <c r="H64" s="8">
         <v>0</v>
       </c>
-      <c r="I64" s="17"/>
-      <c r="J64" s="17"/>
-    </row>
-    <row r="65" ht="28.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A65" s="23" t="s">
+    </row>
+    <row r="65" ht="28.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A65" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B65" s="24"/>
-      <c r="C65" s="24"/>
-      <c r="D65" s="24"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="24"/>
-      <c r="G65" s="24"/>
-      <c r="H65" s="25"/>
-    </row>
-    <row r="66" ht="42.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A66" s="26" t="str">
+      <c r="B65" s="23"/>
+      <c r="C65" s="23"/>
+      <c r="D65" s="23"/>
+      <c r="E65" s="23"/>
+      <c r="F65" s="23"/>
+      <c r="G65" s="23"/>
+      <c r="H65" s="24"/>
+    </row>
+    <row r="66" ht="42.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A66" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A63</f>
         <v>(1) การผลิตภาชนะ เครื่องประดับ เครื่องมือ อุปกรณ์ หรือเครื่องใช้ต่าง ๆ ด้วยโลหะหรือแร่</v>
       </c>
-      <c r="B66" s="27"/>
-      <c r="C66" s="27"/>
-      <c r="D66" s="28"/>
+      <c r="B66" s="26"/>
+      <c r="C66" s="26"/>
+      <c r="D66" s="27"/>
       <c r="E66" s="8">
         <v>1</v>
       </c>
@@ -1979,14 +1925,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" ht="27.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A67" s="29" t="str">
+    <row r="67" ht="27.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A67" s="28" t="str">
         <f>'[1]รายเก่า รายใหม่'!A64</f>
         <v>(2) การถลุงแร่ การหลอม หรือหล่อโลหะทุกชนิด ยกเว้นกิจการที่ได้รับใบอนุญาต ใน 6 (1)</v>
       </c>
-      <c r="B67" s="30"/>
-      <c r="C67" s="30"/>
-      <c r="D67" s="31"/>
+      <c r="B67" s="29"/>
+      <c r="C67" s="29"/>
+      <c r="D67" s="30"/>
       <c r="E67" s="8">
         <v>0</v>
       </c>
@@ -2000,14 +1946,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" ht="45.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A68" s="26" t="str">
+    <row r="68" ht="45.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A68" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A65</f>
         <v>(3) การกลึง เจาะ เชื่อม ตี ตัด ประสาน รีด หรืออัดโลหะด้วยเครื่องจักร หรือก๊าซ หรือไฟฟ้า ยกเว้นกิจการที่ได้รับใบอนุญาตใน 6 (1)</v>
       </c>
-      <c r="B68" s="27"/>
-      <c r="C68" s="27"/>
-      <c r="D68" s="28"/>
+      <c r="B68" s="26"/>
+      <c r="C68" s="26"/>
+      <c r="D68" s="27"/>
       <c r="E68" s="8">
         <v>7</v>
       </c>
@@ -2021,14 +1967,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" ht="45" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A69" s="26" t="str">
+    <row r="69" ht="45" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A69" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A66</f>
         <v>(4) การเคลือบ ชุบโลหะด้วยตะกั่ว สังกะสี ดีบุก โครเมียม นิกเกิล หรือ โลหะอื่นใด ยกเว้นกิจการที่ได้รับใบอนุญาตใน 6 (1)</v>
       </c>
-      <c r="B69" s="27"/>
-      <c r="C69" s="27"/>
-      <c r="D69" s="28"/>
+      <c r="B69" s="26"/>
+      <c r="C69" s="26"/>
+      <c r="D69" s="27"/>
       <c r="E69" s="8">
         <v>0</v>
       </c>
@@ -2042,14 +1988,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A70" s="29" t="str">
+    <row r="70" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A70" s="28" t="str">
         <f>'[1]รายเก่า รายใหม่'!A67</f>
         <v>(5) การขัด ล้างโลหะด้วยเครื่องจักร หรือสารเคมี ยกเว้นกิจการที่ได้รับใบอนุญาต ใน 6 (1)</v>
       </c>
-      <c r="B70" s="30"/>
-      <c r="C70" s="30"/>
-      <c r="D70" s="31"/>
+      <c r="B70" s="29"/>
+      <c r="C70" s="29"/>
+      <c r="D70" s="30"/>
       <c r="E70" s="8">
         <v>0</v>
       </c>
@@ -2063,7 +2009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A68</f>
         <v>(6) การทำเหมืองแร่ สะสม แยก คัดเลือก หรือล้างแร่</v>
@@ -2083,22 +2029,20 @@
       <c r="H71" s="8">
         <v>0</v>
       </c>
-      <c r="I71" s="17"/>
-      <c r="J71" s="17"/>
-    </row>
-    <row r="72" ht="34.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A72" s="23" t="s">
+    </row>
+    <row r="72" ht="34.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A72" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="B72" s="24"/>
-      <c r="C72" s="24"/>
-      <c r="D72" s="24"/>
-      <c r="E72" s="24"/>
-      <c r="F72" s="24"/>
-      <c r="G72" s="24"/>
-      <c r="H72" s="25"/>
-    </row>
-    <row r="73" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B72" s="23"/>
+      <c r="C72" s="23"/>
+      <c r="D72" s="23"/>
+      <c r="E72" s="23"/>
+      <c r="F72" s="23"/>
+      <c r="G72" s="23"/>
+      <c r="H72" s="24"/>
+    </row>
+    <row r="73" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A73" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A70</f>
         <v>(1) การต่อ ประกอบ เคาะ ปะผุ พ่นสี หรือพ่นสารกันสนิมยานยนต์</v>
@@ -2119,7 +2063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A74" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A71</f>
         <v>(2) การผลิตยานยนต์ เครื่องจักร หรือเครื่องกล</v>
@@ -2140,7 +2084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A75" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A72</f>
         <v>(3) การซ่อม การปรับแต่งเครื่องยนต์ เครื่องจักร เครื่องกล ระบบไฟฟ้า ระบบปรับอากาศ หรืออุปกรณ์ที่เป็นส่วนประกอบของยานยนต์ เครื่องจักร หรือเครื่องกล</v>
@@ -2161,7 +2105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A76" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A73</f>
         <v>(4) การประกอบธุรกิจเกี่ยวกับยานยนต์ เครื่องจักรหรือเครื่องกล ซึ่งมีไว้บริการ หรือจำหน่าย และในการประกอบธุรกิจนั้นมีการซ่อมหรือปรับปรุงยานยนต์ เครื่องจักรหรือเครื่องกล ดังกล่าวด้วย</v>
@@ -2182,7 +2126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A77" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A74</f>
         <v>(5) การล้าง ขัดสี เคลือบสี หรืออัดฉีดยานยนต์</v>
@@ -2203,27 +2147,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A78" s="9" t="s">
         <v>20</v>
       </c>
       <c r="B78" s="10"/>
       <c r="C78" s="10"/>
       <c r="D78" s="11"/>
-      <c r="E78" s="22">
-        <v>1</v>
-      </c>
-      <c r="F78" s="22">
-        <v>0</v>
-      </c>
-      <c r="G78" s="22">
-        <v>1</v>
-      </c>
-      <c r="H78" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E78" s="21">
+        <v>1</v>
+      </c>
+      <c r="F78" s="21">
+        <v>0</v>
+      </c>
+      <c r="G78" s="21">
+        <v>1</v>
+      </c>
+      <c r="H78" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A79" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A76</f>
         <v>(7) การจำหน่าย ซ่อม ปะ เชื่อมยางยานยนต์ หรือตั้งศูนย์ถ่วงล้อ</v>
@@ -2244,7 +2188,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A80" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A77</f>
         <v>(8) การผลิต ซ่อม ประกอบ หรืออัดผ้าเบรก ผ้าคลัตช์</v>
@@ -2265,7 +2209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A81" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A78</f>
         <v>(9) การสะสม การซ่อมเครื่องกล เครื่องจักรเก่าหรืออุปกรณ์ที่เป็นส่วนประกอบ ของยานยนต์ เครื่องจักร หรือเครื่องกลเก่า</v>
@@ -2285,24 +2229,21 @@
       <c r="H81" s="8">
         <v>0</v>
       </c>
-      <c r="I81" s="17"/>
-      <c r="J81" s="17"/>
-      <c r="L81" s="32"/>
-    </row>
-    <row r="82" ht="27.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A82" s="23" t="str">
+    </row>
+    <row r="82" ht="27.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A82" s="22" t="str">
         <f>'[1]รายเก่า รายใหม่'!A79</f>
         <v>8.กิจการที่เกี่ยวกับไม้หรือกระดาษ</v>
       </c>
-      <c r="B82" s="24"/>
-      <c r="C82" s="24"/>
-      <c r="D82" s="24"/>
-      <c r="E82" s="24"/>
-      <c r="F82" s="24"/>
-      <c r="G82" s="24"/>
-      <c r="H82" s="25"/>
-    </row>
-    <row r="83" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B82" s="23"/>
+      <c r="C82" s="23"/>
+      <c r="D82" s="23"/>
+      <c r="E82" s="23"/>
+      <c r="F82" s="23"/>
+      <c r="G82" s="23"/>
+      <c r="H82" s="24"/>
+    </row>
+    <row r="83" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A83" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A80</f>
         <v>(1) การผลิตไม้ขีดไฟ</v>
@@ -2323,7 +2264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A84" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A81</f>
         <v>(2) การเลื่อย ซอย ขัด ไส เจาะ ขุดร่อง ทำคิ้ว หรือตัดไม้ด้วยเครื่องจักร</v>
@@ -2344,7 +2285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A85" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A82</f>
         <v>(3) การผลิต พ่น ทาสารเคลือบเงา หรือสี แต่งสำเร็จสิ่งของเครื่องใช้ หรือผลิตภัณฑ์จากไม้ หวาย ชานอ้อย</v>
@@ -2365,7 +2306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A86" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A83</f>
         <v>(4) การอบไม้</v>
@@ -2386,7 +2327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A87" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A84</f>
         <v>(5) การผลิต สะสม แบ่งบรรจุธูป</v>
@@ -2407,7 +2348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A88" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A85</f>
         <v>(6) การผลิตสิ่งของ เครื่องใช้ เครื่องเขียน หรือผลิตภัณฑ์อื่นใดด้วยกระดาษ</v>
@@ -2428,7 +2369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>1</v>
       </c>
@@ -2442,7 +2383,7 @@
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
     </row>
-    <row r="90" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -2460,7 +2401,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A91" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A86</f>
         <v>(7) การผลิตกระดาษชนิดต่าง ๆ</v>
@@ -2481,7 +2422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A92" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A87</f>
         <v>(8) การเผาถ่าน หรือสะสมถ่าน</v>
@@ -2501,30 +2442,28 @@
       <c r="H92" s="8">
         <v>0</v>
       </c>
-      <c r="I92" s="17"/>
-      <c r="J92" s="17"/>
-    </row>
-    <row r="93" ht="29.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A93" s="23" t="str">
+    </row>
+    <row r="93" ht="29.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A93" s="22" t="str">
         <f>'[1]รายเก่า รายใหม่'!A88</f>
         <v>9.กิจการที่เกี่ยวกับการบริการ</v>
       </c>
-      <c r="B93" s="24"/>
-      <c r="C93" s="24"/>
-      <c r="D93" s="24"/>
-      <c r="E93" s="24"/>
-      <c r="F93" s="24"/>
-      <c r="G93" s="24"/>
-      <c r="H93" s="25"/>
-    </row>
-    <row r="94" ht="42.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A94" s="26" t="str">
+      <c r="B93" s="23"/>
+      <c r="C93" s="23"/>
+      <c r="D93" s="23"/>
+      <c r="E93" s="23"/>
+      <c r="F93" s="23"/>
+      <c r="G93" s="23"/>
+      <c r="H93" s="24"/>
+    </row>
+    <row r="94" ht="42.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A94" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A89</f>
         <v>(1) การประกอบกิจการสปาเพื่อสุขภาพ เว้นแต่เป็นการให้บริการในสถานพยาบาล ตามกฎหมายว่าด้วยสถานพยาบาล</v>
       </c>
-      <c r="B94" s="27"/>
-      <c r="C94" s="27"/>
-      <c r="D94" s="28"/>
+      <c r="B94" s="26"/>
+      <c r="C94" s="26"/>
+      <c r="D94" s="27"/>
       <c r="E94" s="8">
         <v>0</v>
       </c>
@@ -2538,7 +2477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A95" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A90</f>
         <v>(2) การประกอบกิจการอาบ อบ นวด</v>
@@ -2559,14 +2498,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" ht="47.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A96" s="26" t="str">
+    <row r="96" ht="47.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A96" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A91</f>
         <v>(3) การประกอบกิจการนวดเพื่อสุขภาพ เว้นแต่เป็นการให้บริการที่ได้รับใบอนุญาตใน 9 (1) หรือในสถานพยาบาลตามกฎหมายว่าด้วยสถานพยาบาล</v>
       </c>
-      <c r="B96" s="27"/>
-      <c r="C96" s="27"/>
-      <c r="D96" s="28"/>
+      <c r="B96" s="26"/>
+      <c r="C96" s="26"/>
+      <c r="D96" s="27"/>
       <c r="E96" s="8">
         <v>0</v>
       </c>
@@ -2580,14 +2519,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" ht="60" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A97" s="26" t="str">
+    <row r="97" ht="60" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A97" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A92</f>
         <v>(4) การประกอบกิจการสถานที่อาบน้ำ อบไอน้ำ อบสมุนไพร เว้นแต่เป็น การให้บริการที่ได้รับใบอนุญาตใน 9 (1) หรือในสถานพยาบาลตามกฎหมายว่าด้วยสถานพยาบาล</v>
       </c>
-      <c r="B97" s="27"/>
-      <c r="C97" s="27"/>
-      <c r="D97" s="28"/>
+      <c r="B97" s="26"/>
+      <c r="C97" s="26"/>
+      <c r="D97" s="27"/>
       <c r="E97" s="8">
         <v>0</v>
       </c>
@@ -2601,14 +2540,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" ht="63.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A98" s="26" t="str">
+    <row r="98" ht="63.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A98" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A93</f>
         <v>(5) การประกอบกิจการโรงแรม สถานที่พักที่มิใช่โรงแรมที่จัดไว้เพื่อให้บริการ พักชั่วคราวสำหรับคนเดินทางหรือบุคคลอื่นใดโดยมีค่าตอบแทน หรือกิจการอื่นในทำนองเดียวกัน</v>
       </c>
-      <c r="B98" s="27"/>
-      <c r="C98" s="27"/>
-      <c r="D98" s="28"/>
+      <c r="B98" s="26"/>
+      <c r="C98" s="26"/>
+      <c r="D98" s="27"/>
       <c r="E98" s="8">
         <v>1</v>
       </c>
@@ -2622,14 +2561,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" ht="44.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A99" s="26" t="str">
+    <row r="99" ht="44.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A99" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A94</f>
         <v>(6) การประกอบกิจการหอพัก อาคารชุดให้เช่า ห้องเช่า หรือห้องแบ่งเช่า หรือกิจการอื่นในทำนองเดียวกัน</v>
       </c>
-      <c r="B99" s="27"/>
-      <c r="C99" s="27"/>
-      <c r="D99" s="28"/>
+      <c r="B99" s="26"/>
+      <c r="C99" s="26"/>
+      <c r="D99" s="27"/>
       <c r="E99" s="8">
         <v>40</v>
       </c>
@@ -2643,7 +2582,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="100" ht="24.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="24.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A100" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A95</f>
         <v>(7) การประกอบกิจการโรงมหรสพ</v>
@@ -2664,14 +2603,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" ht="44.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A101" s="26" t="str">
+    <row r="101" ht="44.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A101" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A96</f>
         <v>(8) การจัดให้มีมหรสพ การแสดงดนตรี เต้นรำ รำวง รองเง็ง ดิสโกเทก คาราโอเกะ หรือตู้เพลง หรือการแสดงอื่น ๆ ในทำนองเดียวกัน</v>
       </c>
-      <c r="B101" s="27"/>
-      <c r="C101" s="27"/>
-      <c r="D101" s="28"/>
+      <c r="B101" s="26"/>
+      <c r="C101" s="26"/>
+      <c r="D101" s="27"/>
       <c r="E101" s="8">
         <v>2</v>
       </c>
@@ -2685,14 +2624,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" ht="43.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A102" s="26" t="str">
+    <row r="102" ht="43.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A102" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A97</f>
         <v>(9) การประกอบกิจการสระว่ายน้ำ หรือกิจการอื่น ๆ ในทำนองเดียวกัน เว้นแต่ เป็นการให้บริการที่ได้รับใบอนุญาตใน 9 (1)</v>
       </c>
-      <c r="B102" s="27"/>
-      <c r="C102" s="27"/>
-      <c r="D102" s="28"/>
+      <c r="B102" s="26"/>
+      <c r="C102" s="26"/>
+      <c r="D102" s="27"/>
       <c r="E102" s="8">
         <v>0</v>
       </c>
@@ -2706,14 +2645,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" ht="41.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A103" s="26" t="str">
+    <row r="103" ht="41.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A103" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A98</f>
         <v>(10) การประกอบกิจการการเล่นสเกต หรือโรลเลอร์เบลด หรือการเล่นอื่น ๆในทำนองเดียวกัน</v>
       </c>
-      <c r="B103" s="27"/>
-      <c r="C103" s="27"/>
-      <c r="D103" s="28"/>
+      <c r="B103" s="26"/>
+      <c r="C103" s="26"/>
+      <c r="D103" s="27"/>
       <c r="E103" s="8">
         <v>0</v>
       </c>
@@ -2727,14 +2666,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" ht="40.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A104" s="26" t="str">
+    <row r="104" ht="40.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A104" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A99</f>
         <v>(11) การประกอบกิจการเสริมสวย หรือแต่งผมเว้นแต่กิจการที่อยู่ในบังคับตามกฎหมายว่าด้วยการประกอบวิชาชีพเวชกรรม</v>
       </c>
-      <c r="B104" s="27"/>
-      <c r="C104" s="27"/>
-      <c r="D104" s="28"/>
+      <c r="B104" s="26"/>
+      <c r="C104" s="26"/>
+      <c r="D104" s="27"/>
       <c r="E104" s="8">
         <v>43</v>
       </c>
@@ -2748,7 +2687,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="105" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A105" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A100</f>
         <v>(12) การประกอบกิจการสถานที่ออกกำลังกาย</v>
@@ -2769,7 +2708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A106" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A101</f>
         <v>(13) การประกอบกิจการให้บริการควบคุมน้ำหนัก</v>
@@ -2786,11 +2725,11 @@
       <c r="G106" s="8">
         <v>0</v>
       </c>
-      <c r="H106" s="17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="H106" s="31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A107" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A102</f>
         <v>(14) การประกอบกิจการสวนสนุก โบว์ลิ่ง หรือตู้เกม</v>
@@ -2811,7 +2750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A108" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A103</f>
         <v>(15) การประกอบกิจการให้บริการคอมพิวเตอร์</v>
@@ -2832,7 +2771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A109" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A104</f>
         <v>(16) การประกอบกิจการสนามกอล์ฟ หรือสนามฝึกซ้อมกอล์ฟ</v>
@@ -2853,14 +2792,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" ht="42" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A110" s="26" t="str">
+    <row r="110" ht="42" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A110" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A105</f>
         <v>(17) การประกอบกิจการห้องปฏิบัติการทางการแพทย์ การสาธารณสุข วิทยาศาสตร์หรือสิ่งแวดล้อม</v>
       </c>
-      <c r="B110" s="27"/>
-      <c r="C110" s="27"/>
-      <c r="D110" s="28"/>
+      <c r="B110" s="26"/>
+      <c r="C110" s="26"/>
+      <c r="D110" s="27"/>
       <c r="E110" s="8">
         <v>0</v>
       </c>
@@ -2874,7 +2813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="111" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A111" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A106</f>
         <v>(18) การประกอบกิจการสักผิวหนัง หรือเจาะส่วนหนึ่งส่วนใดของร่างกาย</v>
@@ -2895,7 +2834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="112" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A112" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A107</f>
         <v>(19) การประกอบกิจการให้บริการเลี้ยงและดูแลเด็กที่บ้านของผู้รับบริการ</v>
@@ -2915,12 +2854,8 @@
       <c r="H112" s="8">
         <v>0</v>
       </c>
-      <c r="I112" s="17"/>
-      <c r="J112" s="17"/>
-      <c r="K112" s="17"/>
-      <c r="L112" s="17"/>
-    </row>
-    <row r="113" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="113" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
         <v>1</v>
       </c>
@@ -2934,7 +2869,7 @@
       <c r="G113" s="3"/>
       <c r="H113" s="3"/>
     </row>
-    <row r="114" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="114" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -2952,7 +2887,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="115" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A115" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A108</f>
         <v>(20) การประกอบกิจการให้บริการดูแลผู้สูงอายุที่บ้านของผู้รับบริการ</v>
@@ -2973,14 +2908,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" ht="44.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A116" s="26" t="str">
+    <row r="116" ht="44.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A116" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A109</f>
         <v>(21) การประกอบกิจการให้บริการสปา อาบน้ำ ตัดขน รับเลี้ยงหรือรับฝากสัตว์ชั่วคราว</v>
       </c>
-      <c r="B116" s="27"/>
-      <c r="C116" s="27"/>
-      <c r="D116" s="28"/>
+      <c r="B116" s="26"/>
+      <c r="C116" s="26"/>
+      <c r="D116" s="27"/>
       <c r="E116" s="8">
         <v>0</v>
       </c>
@@ -2994,20 +2929,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" ht="29.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A117" s="23" t="str">
+    <row r="117" ht="29.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A117" s="22" t="str">
         <f>'[1]รายเก่า รายใหม่'!A110</f>
         <v>10.กิจการที่เกี่ยวกับสิ่งทอ</v>
       </c>
-      <c r="B117" s="24"/>
-      <c r="C117" s="24"/>
-      <c r="D117" s="24"/>
-      <c r="E117" s="24"/>
-      <c r="F117" s="24"/>
-      <c r="G117" s="24"/>
-      <c r="H117" s="25"/>
-    </row>
-    <row r="118" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B117" s="23"/>
+      <c r="C117" s="23"/>
+      <c r="D117" s="23"/>
+      <c r="E117" s="23"/>
+      <c r="F117" s="23"/>
+      <c r="G117" s="23"/>
+      <c r="H117" s="24"/>
+    </row>
+    <row r="118" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A118" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A111</f>
         <v>(1) การปั่นด้าย กรอด้าย ทอผ้าด้วยเครื่องจักร หรือทอผ้าด้วยกี่กระตุก</v>
@@ -3028,7 +2963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="119" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A119" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A112</f>
         <v>(2) การสะสมปอ ป่าน ฝ้าย นุ่น หรือใยสังเคราะห์</v>
@@ -3049,7 +2984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="120" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A120" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A113</f>
         <v>(3) การปั่นฝ้าย นุ่น ใยสังเคราะห์ด้วยเครื่องจักร</v>
@@ -3070,7 +3005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="121" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A121" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A114</f>
         <v>(4) การทอเสื่อ กระสอบ พรม หรือสิ่งทออื่น ๆ ด้วยเครื่องจักร</v>
@@ -3091,7 +3026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="122" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A122" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A115</f>
         <v>(5) การเย็บ ปักผ้า หรือสิ่งทออื่น ๆ ด้วยเครื่องจักร</v>
@@ -3112,7 +3047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="123" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A123" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A116</f>
         <v>(6) การพิมพ์ผ้า และสิ่งทออื่น ๆ</v>
@@ -3133,7 +3068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="124" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A124" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A117</f>
         <v>(7) การซัก อบ รีด หรืออัดกลีบผ้าด้วยเครื่องจักร</v>
@@ -3141,20 +3076,20 @@
       <c r="B124" s="10"/>
       <c r="C124" s="10"/>
       <c r="D124" s="11"/>
-      <c r="E124" s="22">
+      <c r="E124" s="21">
         <v>8</v>
       </c>
-      <c r="F124" s="22">
-        <v>1</v>
-      </c>
-      <c r="G124" s="22">
+      <c r="F124" s="21">
+        <v>1</v>
+      </c>
+      <c r="G124" s="21">
         <v>6</v>
       </c>
-      <c r="H124" s="22">
+      <c r="H124" s="21">
         <v>2</v>
       </c>
     </row>
-    <row r="125" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="125" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A125" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A118</f>
         <v>(8) การย้อม ฟอก กัดสีผ้าหรือสิ่งทออื่น ๆ</v>
@@ -3174,25 +3109,21 @@
       <c r="H125" s="8">
         <v>0</v>
       </c>
-      <c r="I125" s="17"/>
-      <c r="J125" s="17"/>
-      <c r="K125" s="17"/>
-      <c r="L125" s="17"/>
-    </row>
-    <row r="126" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A126" s="23" t="str">
+    </row>
+    <row r="126" ht="31.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A126" s="22" t="str">
         <f>'[1]รายเก่า รายใหม่'!A119</f>
         <v>11.กิจการที่เกี่ยวกับหิน ดิน ทราย ซีเมนต์ หรือวัตถุที่คล้ายคลึง</v>
       </c>
-      <c r="B126" s="24"/>
-      <c r="C126" s="24"/>
-      <c r="D126" s="24"/>
-      <c r="E126" s="24"/>
-      <c r="F126" s="24"/>
-      <c r="G126" s="24"/>
-      <c r="H126" s="25"/>
-    </row>
-    <row r="127" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B126" s="23"/>
+      <c r="C126" s="23"/>
+      <c r="D126" s="23"/>
+      <c r="E126" s="23"/>
+      <c r="F126" s="23"/>
+      <c r="G126" s="23"/>
+      <c r="H126" s="24"/>
+    </row>
+    <row r="127" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A127" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A120</f>
         <v>(1) การผลิตภาชนะดินเผาหรือผลิตภัณฑ์ดินเผา</v>
@@ -3213,7 +3144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="128" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A128" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A121</f>
         <v>(2) การระเบิด โม่ บด หรือย่อยหิน ด้วยเครื่องจักร</v>
@@ -3221,20 +3152,20 @@
       <c r="B128" s="10"/>
       <c r="C128" s="10"/>
       <c r="D128" s="11"/>
-      <c r="E128" s="22">
-        <v>0</v>
-      </c>
-      <c r="F128" s="22">
-        <v>0</v>
-      </c>
-      <c r="G128" s="22">
-        <v>0</v>
-      </c>
-      <c r="H128" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E128" s="21">
+        <v>0</v>
+      </c>
+      <c r="F128" s="21">
+        <v>0</v>
+      </c>
+      <c r="G128" s="21">
+        <v>0</v>
+      </c>
+      <c r="H128" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A129" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A122</f>
         <v>(3) การผลิตสิ่งของ เครื่องใช้หรือผลิตภัณฑ์อื่น ๆ ด้วยซีเมนต์ หรือวัตถุที่คล้ายคลึง</v>
@@ -3255,14 +3186,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" ht="45.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A130" s="26" t="str">
+    <row r="130" ht="45.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A130" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A123</f>
         <v>(4) การสะสม ผสมซีเมนต์ หิน ดิน ทราย วัสดุก่อสร้าง รวมทั้งการขุด ตัก ดูด โม่ บด หรือย่อย ด้วยเครื่องจักร ยกเว้นกิจการที่ได้รับใบอนุญาตใน 11 (2)</v>
       </c>
-      <c r="B130" s="27"/>
-      <c r="C130" s="27"/>
-      <c r="D130" s="28"/>
+      <c r="B130" s="26"/>
+      <c r="C130" s="26"/>
+      <c r="D130" s="27"/>
       <c r="E130" s="8">
         <v>17</v>
       </c>
@@ -3276,7 +3207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="131" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A131" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A124</f>
         <v>(5) การเจียระไนเพชร พลอย หิน หรือกระจก หรือวัตถุที่คล้ายคลึง</v>
@@ -3284,20 +3215,20 @@
       <c r="B131" s="10"/>
       <c r="C131" s="10"/>
       <c r="D131" s="11"/>
-      <c r="E131" s="22">
-        <v>0</v>
-      </c>
-      <c r="F131" s="22">
-        <v>0</v>
-      </c>
-      <c r="G131" s="22">
-        <v>0</v>
-      </c>
-      <c r="H131" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E131" s="21">
+        <v>0</v>
+      </c>
+      <c r="F131" s="21">
+        <v>0</v>
+      </c>
+      <c r="G131" s="21">
+        <v>0</v>
+      </c>
+      <c r="H131" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A132" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A125</f>
         <v>(6) การเลื่อย ตัด หรือประดิษฐ์หินเป็นสิ่งของ เครื่องใช้ หรือผลิตภัณฑ์ต่าง ๆ</v>
@@ -3305,20 +3236,20 @@
       <c r="B132" s="10"/>
       <c r="C132" s="10"/>
       <c r="D132" s="11"/>
-      <c r="E132" s="22">
-        <v>0</v>
-      </c>
-      <c r="F132" s="22">
-        <v>0</v>
-      </c>
-      <c r="G132" s="22">
-        <v>0</v>
-      </c>
-      <c r="H132" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E132" s="21">
+        <v>0</v>
+      </c>
+      <c r="F132" s="21">
+        <v>0</v>
+      </c>
+      <c r="G132" s="21">
+        <v>0</v>
+      </c>
+      <c r="H132" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A133" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A126</f>
         <v>(7) การผลิตชอล์ก ปูนปลาสเตอร์ ปูนขาว ดินสอพอง หรือเผาหินปูน</v>
@@ -3326,20 +3257,20 @@
       <c r="B133" s="10"/>
       <c r="C133" s="10"/>
       <c r="D133" s="11"/>
-      <c r="E133" s="22">
-        <v>0</v>
-      </c>
-      <c r="F133" s="22">
-        <v>0</v>
-      </c>
-      <c r="G133" s="22">
-        <v>0</v>
-      </c>
-      <c r="H133" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E133" s="21">
+        <v>0</v>
+      </c>
+      <c r="F133" s="21">
+        <v>0</v>
+      </c>
+      <c r="G133" s="21">
+        <v>0</v>
+      </c>
+      <c r="H133" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A134" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A127</f>
         <v>(8) การผลิตผลิตภัณฑ์ต่าง ๆ ที่มีแร่ใยหินเป็นส่วนประกอบหรือส่วนผสม</v>
@@ -3347,20 +3278,20 @@
       <c r="B134" s="10"/>
       <c r="C134" s="10"/>
       <c r="D134" s="11"/>
-      <c r="E134" s="22">
-        <v>0</v>
-      </c>
-      <c r="F134" s="22">
-        <v>0</v>
-      </c>
-      <c r="G134" s="22">
-        <v>0</v>
-      </c>
-      <c r="H134" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E134" s="21">
+        <v>0</v>
+      </c>
+      <c r="F134" s="21">
+        <v>0</v>
+      </c>
+      <c r="G134" s="21">
+        <v>0</v>
+      </c>
+      <c r="H134" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A135" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A128</f>
         <v>(9) การผลิต ตัด บดกระจกหรือผลิตภัณฑ์แก้ว</v>
@@ -3368,20 +3299,20 @@
       <c r="B135" s="10"/>
       <c r="C135" s="10"/>
       <c r="D135" s="11"/>
-      <c r="E135" s="22">
-        <v>0</v>
-      </c>
-      <c r="F135" s="22">
-        <v>0</v>
-      </c>
-      <c r="G135" s="22">
-        <v>0</v>
-      </c>
-      <c r="H135" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E135" s="21">
+        <v>0</v>
+      </c>
+      <c r="F135" s="21">
+        <v>0</v>
+      </c>
+      <c r="G135" s="21">
+        <v>0</v>
+      </c>
+      <c r="H135" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A136" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A129</f>
         <v>(10) การผลิตกระดาษทราย หรือผ้าทราย</v>
@@ -3389,20 +3320,20 @@
       <c r="B136" s="10"/>
       <c r="C136" s="10"/>
       <c r="D136" s="11"/>
-      <c r="E136" s="22">
-        <v>0</v>
-      </c>
-      <c r="F136" s="22">
-        <v>0</v>
-      </c>
-      <c r="G136" s="22">
-        <v>0</v>
-      </c>
-      <c r="H136" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="E136" s="21">
+        <v>0</v>
+      </c>
+      <c r="F136" s="21">
+        <v>0</v>
+      </c>
+      <c r="G136" s="21">
+        <v>0</v>
+      </c>
+      <c r="H136" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A137" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A130</f>
         <v>(11) การผลิตใยแก้ว หรือผลิตภัณฑ์จากใยแก้ว</v>
@@ -3410,27 +3341,27 @@
       <c r="B137" s="10"/>
       <c r="C137" s="10"/>
       <c r="D137" s="11"/>
-      <c r="E137" s="22">
-        <v>0</v>
-      </c>
-      <c r="F137" s="22">
-        <v>0</v>
-      </c>
-      <c r="G137" s="22">
-        <v>0</v>
-      </c>
-      <c r="H137" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" ht="42.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A138" s="26" t="str">
+      <c r="E137" s="21">
+        <v>0</v>
+      </c>
+      <c r="F137" s="21">
+        <v>0</v>
+      </c>
+      <c r="G137" s="21">
+        <v>0</v>
+      </c>
+      <c r="H137" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" ht="42.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A138" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A131</f>
         <v>(12) การล้าง การขัดด้วยการพ่นทรายลงบนพื้นผิวกระจก แก้ว หิน หรือวัตถุอื่นใด ยกเว้นกิจการที่ได้รับใบอนุญาตใน 6 (5)</v>
       </c>
-      <c r="B138" s="27"/>
-      <c r="C138" s="27"/>
-      <c r="D138" s="28"/>
+      <c r="B138" s="26"/>
+      <c r="C138" s="26"/>
+      <c r="D138" s="27"/>
       <c r="E138" s="8">
         <v>0</v>
       </c>
@@ -3443,30 +3374,28 @@
       <c r="H138" s="8">
         <v>0</v>
       </c>
-      <c r="I138" s="17"/>
-      <c r="J138" s="17"/>
-    </row>
-    <row r="139" ht="30.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A139" s="23" t="str">
+    </row>
+    <row r="139" ht="30.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A139" s="22" t="str">
         <f>'[1]รายเก่า รายใหม่'!A132</f>
         <v>12.กิจการที่เกี่ยวกับปิโตรเลียม ปิโตรเคมี ถ่านหิน ถ่านโค้ก และสารเคมีต่าง ๆ</v>
       </c>
-      <c r="B139" s="24"/>
-      <c r="C139" s="24"/>
-      <c r="D139" s="24"/>
-      <c r="E139" s="24"/>
-      <c r="F139" s="24"/>
-      <c r="G139" s="24"/>
-      <c r="H139" s="25"/>
-    </row>
-    <row r="140" ht="41.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A140" s="26" t="str">
+      <c r="B139" s="23"/>
+      <c r="C139" s="23"/>
+      <c r="D139" s="23"/>
+      <c r="E139" s="23"/>
+      <c r="F139" s="23"/>
+      <c r="G139" s="23"/>
+      <c r="H139" s="24"/>
+    </row>
+    <row r="140" ht="41.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A140" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A133</f>
         <v>(1) การผลิต สะสม บรรจุ หรือขนส่งกรด ด่าง สารออกซิไดซ์ หรือสารตัวทำละลาย</v>
       </c>
-      <c r="B140" s="27"/>
-      <c r="C140" s="27"/>
-      <c r="D140" s="28"/>
+      <c r="B140" s="26"/>
+      <c r="C140" s="26"/>
+      <c r="D140" s="27"/>
       <c r="E140" s="8">
         <v>2</v>
       </c>
@@ -3480,7 +3409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="141" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A141" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A134</f>
         <v>(2) การผลิต สะสม บรรจุ หรือขนส่งก๊าซ</v>
@@ -3501,7 +3430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="142" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A142" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A135</f>
         <v>(3) การผลิต สะสม กลั่น หรือขนส่งปิโตรเลียมหรือผลิตภัณฑ์ปิโตรเลียม</v>
@@ -3522,7 +3451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="143" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A143" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A136</f>
         <v>(4) การผลิต สะสม หรือขนส่งถ่านหิน หรือถ่านโค้ก</v>
@@ -3543,7 +3472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="144" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A144" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A137</f>
         <v>(5) การพ่นสี ยกเว้นกิจการที่ได้รับใบอนุญาตใน 7 (1)</v>
@@ -3560,14 +3489,11 @@
       <c r="G144" s="8">
         <v>0</v>
       </c>
-      <c r="H144" s="33">
-        <v>0</v>
-      </c>
-      <c r="I144" s="32"/>
-      <c r="J144" s="32"/>
-      <c r="L144" s="34"/>
-    </row>
-    <row r="145" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="H144" s="32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A145" s="3" t="s">
         <v>1</v>
       </c>
@@ -3581,7 +3507,7 @@
       <c r="G145" s="3"/>
       <c r="H145" s="3"/>
     </row>
-    <row r="146" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="146" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
@@ -3599,14 +3525,14 @@
         <v>6</v>
       </c>
     </row>
-    <row r="147" ht="40.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A147" s="26" t="str">
+    <row r="147" ht="40.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A147" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A138</f>
         <v>(6) การผลิตสิ่งของเครื่องใช้หรือผลิตภัณฑ์ด้วยยางเทียม พลาสติก เซลลูลอยด์ เบเกอร์ไลท์ หรือวัตถุที่คล้ายคลึง</v>
       </c>
-      <c r="B147" s="27"/>
-      <c r="C147" s="27"/>
-      <c r="D147" s="28"/>
+      <c r="B147" s="26"/>
+      <c r="C147" s="26"/>
+      <c r="D147" s="27"/>
       <c r="E147" s="8">
         <v>0</v>
       </c>
@@ -3620,7 +3546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="148" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A148" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A139</f>
         <v>(7) การโม่ สะสม หรือบดชัน</v>
@@ -3640,9 +3566,8 @@
       <c r="H148" s="8">
         <v>0</v>
       </c>
-      <c r="M148" s="35"/>
-    </row>
-    <row r="149" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A149" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A140</f>
         <v>(8) การผลิตสีหรือน้ำมนผสมสี</v>
@@ -3663,7 +3588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="150" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A150" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A141</f>
         <v>(9) การผลิต ล้างฟิล์มรูปถ่ายหรือฟิล์มภาพยนตร์</v>
@@ -3684,14 +3609,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" ht="40.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A151" s="26" t="str">
+    <row r="151" ht="40.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A151" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A142</f>
         <v>(10) การเคลือบ ชุบวัตถุด้วยพลาสติก เซลลูลอยด์ เบเกอร์ไลท์ หรือวัตถุที่คล้ายคลึง</v>
       </c>
-      <c r="B151" s="27"/>
-      <c r="C151" s="27"/>
-      <c r="D151" s="28"/>
+      <c r="B151" s="26"/>
+      <c r="C151" s="26"/>
+      <c r="D151" s="27"/>
       <c r="E151" s="8">
         <v>0</v>
       </c>
@@ -3705,7 +3630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="152" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A152" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A143</f>
         <v>(11) การผลิตพลาสติก เซลลูลอยด์ เบเกอร์ไลท์ หรือวัตถุที่คล้ายคลึง</v>
@@ -3726,7 +3651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="153" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A153" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A144</f>
         <v>(12) การผลิต หรือบรรจุสารเคมีดับเพลิง</v>
@@ -3747,7 +3672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="154" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A154" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A145</f>
         <v>(13) การผลิตน้ำแข็งแห้ง</v>
@@ -3768,14 +3693,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" ht="41.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A155" s="26" t="str">
+    <row r="155" ht="41.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A155" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A146</f>
         <v>(14) การผลิต สะสม ขนส่งดอกไม้เพลิง หรือสารเคมีอันเป็นส่วนประกอบในการผลิตดอกไม้เพลิง</v>
       </c>
-      <c r="B155" s="27"/>
-      <c r="C155" s="27"/>
-      <c r="D155" s="28"/>
+      <c r="B155" s="26"/>
+      <c r="C155" s="26"/>
+      <c r="D155" s="27"/>
       <c r="E155" s="8">
         <v>0</v>
       </c>
@@ -3789,7 +3714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="156" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A156" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A147</f>
         <v>(15) การผลิตเชลแล็ก หรือสารเคลือบเงา</v>
@@ -3810,7 +3735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="157" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A157" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A148</f>
         <v>(16) การผลิต สะสม บรรจุ ขนส่งสารกำจัดศัตรูพืชหรือพาหะนำโรค</v>
@@ -3831,7 +3756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="158" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A158" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A149</f>
         <v>(17) การผลิต สะสม หรือบรรจุกาว</v>
@@ -3839,36 +3764,33 @@
       <c r="B158" s="10"/>
       <c r="C158" s="10"/>
       <c r="D158" s="11"/>
-      <c r="E158" s="22">
+      <c r="E158" s="21">
         <v>2</v>
       </c>
-      <c r="F158" s="22">
-        <v>0</v>
-      </c>
-      <c r="G158" s="22">
+      <c r="F158" s="21">
+        <v>0</v>
+      </c>
+      <c r="G158" s="21">
         <v>2</v>
       </c>
-      <c r="H158" s="22">
-        <v>0</v>
-      </c>
-      <c r="I158" s="36"/>
-      <c r="J158" s="36"/>
-      <c r="L158" s="37"/>
-    </row>
-    <row r="159" ht="27.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A159" s="23" t="str">
+      <c r="H158" s="21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" ht="27.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A159" s="22" t="str">
         <f>'[1]รายเก่า รายใหม่'!A150</f>
         <v>13.กิจการอื่น ๆ</v>
       </c>
-      <c r="B159" s="24"/>
-      <c r="C159" s="24"/>
-      <c r="D159" s="24"/>
-      <c r="E159" s="24"/>
-      <c r="F159" s="24"/>
-      <c r="G159" s="24"/>
-      <c r="H159" s="25"/>
-    </row>
-    <row r="160" ht="20.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="B159" s="23"/>
+      <c r="C159" s="23"/>
+      <c r="D159" s="23"/>
+      <c r="E159" s="23"/>
+      <c r="F159" s="23"/>
+      <c r="G159" s="23"/>
+      <c r="H159" s="24"/>
+    </row>
+    <row r="160" ht="20.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A160" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A151</f>
         <v>(1) การพิมพ์หนังสือหรือสิ่งพิมพ์อื่นที่มีลักษณะเดียวกันด้วยเครื่องจักร</v>
@@ -3889,14 +3811,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" ht="45.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A161" s="26" t="str">
+    <row r="161" ht="45.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A161" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A152</f>
         <v>(2) การผลิต ซ่อมเครื่องอิเล็กทรอนิกส์ เครื่องไฟฟ้า อุปกรณ์อิเล็กทรอนิกส์หรืออุปกรณ์ไฟฟ้า</v>
       </c>
-      <c r="B161" s="27"/>
-      <c r="C161" s="27"/>
-      <c r="D161" s="28"/>
+      <c r="B161" s="26"/>
+      <c r="C161" s="26"/>
+      <c r="D161" s="27"/>
       <c r="E161" s="8">
         <v>3</v>
       </c>
@@ -3910,7 +3832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" ht="24.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="162" ht="24.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A162" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A153</f>
         <v>(3) การผลิตเทียน หรือเทียนไข หรือวัตถุที่คล้ายคลึง</v>
@@ -3931,7 +3853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="163" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A163" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A154</f>
         <v>(4) การพิมพ์แบบ พิมพ์เขียว หรือถ่ายเอกสาร</v>
@@ -3952,7 +3874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="164" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A164" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A155</f>
         <v>(5) การสะสมวัตถุหรือสิ่งของที่ชำรุด ใช้แล้วหรือเหลือใช้</v>
@@ -3973,7 +3895,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" ht="29.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="165" ht="29.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A165" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A156</f>
         <v>(6) การประกอบกิจการโกดังสินค้า</v>
@@ -3994,14 +3916,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" ht="39" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A166" s="26" t="str">
+    <row r="166" ht="39" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A166" s="25" t="str">
         <f>'[1]รายเก่า รายใหม่'!A157</f>
         <v>(7) การล้างขวด ภาชนะหรือบรรจุภัณฑ์ที่ใช้แล้วเพื่อนำไปใช้ใหม่หรือแปรสภาพเป็นผลิตภัณฑ์ใหม่</v>
       </c>
-      <c r="B166" s="27"/>
-      <c r="C166" s="27"/>
-      <c r="D166" s="28"/>
+      <c r="B166" s="26"/>
+      <c r="C166" s="26"/>
+      <c r="D166" s="27"/>
       <c r="E166" s="8">
         <v>1</v>
       </c>
@@ -4015,7 +3937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" ht="22.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="167" ht="22.5" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A167" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A158</f>
         <v>(8) การพิมพ์ เขียน พ่นสี หรือวิธีอื่นใดลงบนวัตถุที่มิใช่สิ่งทอ</v>
@@ -4036,7 +3958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" ht="23.25" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="168" ht="23.25" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A168" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A159</f>
         <v>(9) การประกอบกิจการท่าเทียบเรือประมง สะพานปลา หรือแพปลา</v>
@@ -4057,7 +3979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" ht="27.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="169" ht="27.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A169" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A160</f>
         <v>(10) การบรรจุหีบห่อสินค้าโดยใช้เครื่องจักร</v>
@@ -4078,7 +4000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" ht="24.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="170" ht="24.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A170" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A161</f>
         <v>(11) การให้บริการควบคุมป้องกันและกำจัดแมลง หรือสัตว์พาหะนำโรค</v>
@@ -4099,7 +4021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="171" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A171" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A162</f>
         <v>(12) การผลิตสิ่งของ เครื่องใช้ หรือผลิตภัณฑ์จากยาง</v>
@@ -4120,7 +4042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" ht="24" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="172" ht="24" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A172" s="9" t="str">
         <f>'[1]รายเก่า รายใหม่'!A163</f>
         <v>(13) การผลิต สะสม หรือขนส่งไบโอดีเซลและเอทานอล</v>
@@ -4140,32 +4062,28 @@
       <c r="H172" s="8">
         <v>0</v>
       </c>
-      <c r="I172" s="38"/>
-      <c r="J172" s="38"/>
-      <c r="K172" s="38"/>
-      <c r="L172" s="38"/>
-    </row>
-    <row r="173" ht="30.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A173" s="39" t="str">
+    </row>
+    <row r="173" ht="30.75" customHeight="1" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="A173" s="33" t="str">
         <f>'[1]รายเก่า รายใหม่'!A164</f>
         <v>รวม</v>
       </c>
-      <c r="B173" s="40"/>
-      <c r="C173" s="40"/>
-      <c r="D173" s="41"/>
-      <c r="E173" s="42">
+      <c r="B173" s="34"/>
+      <c r="C173" s="34"/>
+      <c r="D173" s="35"/>
+      <c r="E173" s="36">
         <f>SUM(J172+J158+J144+J138+J125+J112+J92+J81+J71+J64+J52+J46+J19)</f>
         <v>303</v>
       </c>
-      <c r="F173" s="42">
+      <c r="F173" s="36">
         <f>SUM(K172+K125+K112+1)</f>
         <v>9</v>
       </c>
-      <c r="G173" s="42">
+      <c r="G173" s="36">
         <f>SUM(I172+I158+I144+I138+I125+I112+I81+I71+I64+I52+I46+I19+I92)</f>
         <v>272</v>
       </c>
-      <c r="H173" s="42">
+      <c r="H173" s="36">
         <f>SUM(L172+L158+L144+L125+L112+L81+K46)</f>
         <v>38</v>
       </c>

</xml_diff>